<commit_message>
New ID code generation
</commit_message>
<xml_diff>
--- a/data/modules/nwss_reporting_to_v2/ids/nwss_reporting_to_v2_id_code.xlsx
+++ b/data/modules/nwss_reporting_to_v2/ids/nwss_reporting_to_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/data/modules/nwss_reporting_to_v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09629C71-B09E-5D45-A69B-03FBFE11312D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CDE0F0A-9FA0-F440-A876-D572634AA2CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="86">
   <si>
     <t>addresses</t>
   </si>
@@ -226,9 +226,6 @@
     <t>dat.protocols.__protocolID</t>
   </si>
   <si>
-    <t>dat.protocolSteps.__stepID</t>
-  </si>
-  <si>
     <t>dat.instruments.instrumentID</t>
   </si>
   <si>
@@ -247,9 +244,6 @@
     <t>dat.sites.__siteID</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.addresses.country, datEmpty.addresses.pCode, datEmpty.addresses.city[:3])</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.organizations.organizationID, datEmpty.contacts.role[:3])</t>
   </si>
   <si>
@@ -271,18 +265,9 @@
     <t>fn.makeid(datEmpty.protocols.name, datEmpty.protocols.protocolVersion)</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.organizations.organizationID, datEmpty.protocolSteps.measure[-3:] if datEmpty.protocolSteps.measure else datEmpty.protocolSteps.method[-3:])</t>
-  </si>
-  <si>
-    <t>datEmpty.qualityReports.__qualityReportID</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.addresses.country, datEmpty.addresses.pCode, datEmpty.addresses.city[:3], datEmpty.sites.name[:3])</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures", "__measureSetRepID", equals=dat.measureSets.__measureSetRepID)))</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.addresses.country, datEmpty.addresses.pCode, datEmpty.addresses.city[:3], f"{fn.rownum:03d}")</t>
   </si>
   <si>
@@ -298,7 +283,16 @@
     <t>fn.datetimetz(dat.samples.__collDT.split('/'))</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.samples.siteID, datEmpty.samples.collDT if datEmpty.samples.collDT else datEmpty.samples.collDTEnd, f"{fn.rownum:03d}")</t>
+    <t>dat.measures.measureRepID</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.organizations.organizationID, datEmpty.protocolSteps.measure[-3:] if dat.protocolSteps.measure else datEmpty.protocolSteps.method[-3:])</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.samples.siteID, datEmpty.samples.collDT if dat.samples.collDT else datEmpty.samples.collDTEnd, f"{fn.rownum:03d}")</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures", "(__source_file_and_row__)", equals=dat.measureSets.get("(__source_file_and_row__)"))))</t>
   </si>
 </sst>
 </file>
@@ -693,10 +687,10 @@
         <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="E2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -721,7 +715,7 @@
         <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -816,10 +810,10 @@
         <v>51</v>
       </c>
       <c r="D18" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E18" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -871,10 +865,10 @@
         <v>53</v>
       </c>
       <c r="D25" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E25" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -973,10 +967,10 @@
         <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="E35" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1023,7 +1017,7 @@
         <v>59</v>
       </c>
       <c r="D40" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1059,7 +1053,10 @@
         <v>61</v>
       </c>
       <c r="D44" t="s">
-        <v>76</v>
+        <v>74</v>
+      </c>
+      <c r="E44" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1095,12 +1092,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>12</v>
       </c>
@@ -1108,7 +1105,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>12</v>
       </c>
@@ -1119,10 +1116,10 @@
         <v>62</v>
       </c>
       <c r="D52" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>12</v>
       </c>
@@ -1133,7 +1130,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>12</v>
       </c>
@@ -1144,7 +1141,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>12</v>
       </c>
@@ -1155,7 +1152,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>14</v>
       </c>
@@ -1163,13 +1160,10 @@
         <v>15</v>
       </c>
       <c r="C57" t="s">
-        <v>63</v>
-      </c>
-      <c r="D57" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>14</v>
       </c>
@@ -1180,7 +1174,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>14</v>
       </c>
@@ -1191,7 +1185,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>14</v>
       </c>
@@ -1199,10 +1193,10 @@
         <v>16</v>
       </c>
       <c r="C60" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>17</v>
       </c>
@@ -1210,13 +1204,10 @@
         <v>18</v>
       </c>
       <c r="C62" t="s">
-        <v>79</v>
-      </c>
-      <c r="D62" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>17</v>
       </c>
@@ -1224,37 +1215,40 @@
         <v>4</v>
       </c>
       <c r="C63" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+      <c r="E63" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>17</v>
       </c>
       <c r="B64" t="s">
         <v>6</v>
       </c>
-      <c r="C64" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E64" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>17</v>
       </c>
       <c r="B65" t="s">
         <v>9</v>
       </c>
-      <c r="C65" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E65" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>19</v>
       </c>
@@ -1262,13 +1256,13 @@
         <v>6</v>
       </c>
       <c r="C69" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D69" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>19</v>
       </c>
@@ -1279,7 +1273,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>19</v>
       </c>
@@ -1290,7 +1284,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>19</v>
       </c>
@@ -1301,7 +1295,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>19</v>
       </c>
@@ -1312,7 +1306,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>19</v>
       </c>
@@ -1323,18 +1317,18 @@
         <v>47</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>19</v>
       </c>
       <c r="B75" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C75" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>20</v>
       </c>
@@ -1342,7 +1336,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>20</v>
       </c>
@@ -1350,13 +1344,13 @@
         <v>8</v>
       </c>
       <c r="C78" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D78" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>20</v>
       </c>
@@ -1367,7 +1361,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>20</v>
       </c>

</xml_diff>

<commit_message>
Updates to ID code
</commit_message>
<xml_diff>
--- a/data/modules/nwss_reporting_to_v2/ids/nwss_reporting_to_v2_id_code.xlsx
+++ b/data/modules/nwss_reporting_to_v2/ids/nwss_reporting_to_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/data/modules/nwss_reporting_to_v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CDE0F0A-9FA0-F440-A876-D572634AA2CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{494ADC81-BD65-DF45-AAB2-E684E26B4CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="87">
   <si>
     <t>addresses</t>
   </si>
@@ -293,6 +293,9 @@
   </si>
   <si>
     <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures", "(__source_file_and_row__)", equals=dat.measureSets.get("(__source_file_and_row__)"))))</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.addresses.country, datEmpty.addresses.pCode, datEmpty.addresses.city[:3])</t>
   </si>
 </sst>
 </file>
@@ -687,7 +690,7 @@
         <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="E2" t="s">
         <v>77</v>

</xml_diff>